<commit_message>
feat: _common 的 n_default 加「交易」選項（條件 trade 事實＝role.json trade:true），所有商人自動有，karen/xi 的 choice:n_default 拿掉；COM_Talk 條件附帶 NPC 情境事實
</commit_message>
<xml_diff>
--- a/xls/dialog.xlsx
+++ b/xls/dialog.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="62">
   <si>
     <t>#</t>
   </si>
@@ -114,6 +114,12 @@
     <t>close</t>
   </si>
   <si>
+    <t>交易</t>
+  </si>
+  <si>
+    <t>trade</t>
+  </si>
+  <si>
     <t>聊天</t>
   </si>
   <si>
@@ -196,15 +202,6 @@
   </si>
   <si>
     <t>!_first_meet</t>
-  </si>
-  <si>
-    <t>choice:n_default</t>
-  </si>
-  <si>
-    <t>交易</t>
-  </si>
-  <si>
-    <t>trade</t>
   </si>
   <si>
     <t>很高興認識你，我是Xi</t>
@@ -650,7 +647,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" defaultColWidth="9" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="3.86" customWidth="1"/>
@@ -953,16 +950,16 @@
         <v>9</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="G15" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="H15" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="H15" s="9" t="s">
-        <v>9</v>
-      </c>
       <c r="I15" s="9">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -976,93 +973,95 @@
         <v>9</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E16" s="9" t="s">
         <v>9</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="G16" s="9" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="H16" s="9" t="s">
         <v>9</v>
       </c>
       <c r="I16" s="9">
-        <v>99</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C17" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="E17" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="F17" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="11"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>9</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D19" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E19" s="9" t="s">
+      <c r="B17" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="G17" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="H17" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="I17" s="9">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="9"/>
+      <c r="C18" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>9</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="G20" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="H20" s="9" t="s">
-        <v>38</v>
-      </c>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
       <c r="I20" s="9"/>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -1076,19 +1075,19 @@
         <v>9</v>
       </c>
       <c r="D21" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="G21" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="E21" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="F21" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="G21" s="9" t="s">
+      <c r="H21" s="9" t="s">
         <v>40</v>
-      </c>
-      <c r="H21" s="9" t="s">
-        <v>41</v>
       </c>
       <c r="I21" s="9"/>
     </row>
@@ -1103,19 +1102,19 @@
         <v>9</v>
       </c>
       <c r="D22" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="G22" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="E22" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="F22" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="G22" s="9" t="s">
+      <c r="H22" s="9" t="s">
         <v>43</v>
-      </c>
-      <c r="H22" s="9" t="s">
-        <v>44</v>
       </c>
       <c r="I22" s="9"/>
     </row>
@@ -1130,19 +1129,19 @@
         <v>9</v>
       </c>
       <c r="D23" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="G23" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="E23" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="G23" s="9" t="s">
+      <c r="H23" s="9" t="s">
         <v>46</v>
-      </c>
-      <c r="H23" s="9" t="s">
-        <v>47</v>
       </c>
       <c r="I23" s="9"/>
     </row>
@@ -1150,51 +1149,53 @@
       <c r="A24" t="s">
         <v>9</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="B24" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="C24" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="D24" s="11" t="s">
+      <c r="C24" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="G24" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="E24" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="F24" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="G24" s="11" t="s">
+      <c r="H24" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="I24" s="9"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>9</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D25" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="E25" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="F25" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="G25" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="H24" s="11"/>
-      <c r="I24" s="11"/>
-    </row>
-    <row r="26" ht="94.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>9</v>
-      </c>
-      <c r="B26" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="C26" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D26" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E26" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="F26" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="G26" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="H26" s="9"/>
-      <c r="I26" s="9"/>
+      <c r="H25" s="11"/>
+      <c r="I25" s="11"/>
     </row>
     <row r="27" ht="94.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
@@ -1204,7 +1205,7 @@
         <v>24</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D27" s="9" t="s">
         <v>9</v>
@@ -1216,12 +1217,12 @@
         <v>52</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H27" s="9"/>
       <c r="I27" s="9"/>
     </row>
-    <row r="28" ht="110.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" ht="94.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>9</v>
       </c>
@@ -1229,7 +1230,7 @@
         <v>24</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D28" s="9" t="s">
         <v>9</v>
@@ -1241,45 +1242,70 @@
         <v>54</v>
       </c>
       <c r="G28" s="9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H28" s="9"/>
       <c r="I28" s="9"/>
     </row>
-    <row r="29" ht="126" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" ht="110.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>9</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C29" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="D29" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="E29" s="11" t="s">
+      <c r="C29" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E29" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="F29" s="11" t="s">
+      <c r="F29" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="G29" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="H29" s="11"/>
-      <c r="I29" s="11"/>
+      <c r="G29" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="H29" s="9"/>
+      <c r="I29" s="9"/>
+    </row>
+    <row r="30" ht="126" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>9</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C30" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D30" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="E30" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="F30" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="G30" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="H30" s="11"/>
+      <c r="I30" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" defaultColWidth="9" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="3.86" customWidth="1"/>
@@ -1335,7 +1361,7 @@
         <v>9</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>9</v>
@@ -1344,48 +1370,19 @@
         <v>9</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I2" s="7"/>
-    </row>
-    <row r="4" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="G4" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="H4" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="I4" s="11">
-        <v>10</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" defaultColWidth="9" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="3.86" customWidth="1"/>
@@ -1441,7 +1438,7 @@
         <v>9</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>9</v>
@@ -1450,41 +1447,12 @@
         <v>9</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I2" s="7"/>
-    </row>
-    <row r="4" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="G4" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="H4" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="I4" s="11">
-        <v>10</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>